<commit_message>
chore(fixtures): split villanos sample into week1 and week2 excel files
Update the sample excel generator and fixtures so villanos test data publishes one dienst pattern per week, avoiding same-day double dienst confusion during mobile agenda validation.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ambulancias-goruiz-backend/fixtures/sample-excel-villanos.xlsx
+++ b/ambulancias-goruiz-backend/fixtures/sample-excel-villanos.xlsx
@@ -401,7 +401,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>VILLANOS SA — 1.ª semana: 20.04–26.04.2026 | weekStart 2026-04-20 | Pareja 0001+0002 (García / Soto) — Lu–V</v>
+        <v>VILLANOS SA — 1.ª semana: 20.04–26.04.2026 | weekStart 2026-04-20 | SOLO Dienst Früh | Pareja 0001+0002 (García / Soto) — Lu–V</v>
       </c>
       <c r="B1" t="str">
         <v/>
@@ -511,52 +511,27 @@
         <v/>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
+    <row r="4">
       <c r="A4" t="str">
         <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>Nacht — pareja 0001+0002</v>
-      </c>
-      <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">20:00-08:00
-NEF-2
-0001
-García, L.
-Soto, M.
-0002</v>
-      </c>
-      <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">20:00-08:00
-NEF-2
-0002
-Soto, M.
-García, L.
-0001</v>
-      </c>
-      <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">20:00-08:00
-NEF-2
-0001
-García, L.
-Soto, M.
-0002</v>
-      </c>
-      <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">20:00-08:00
-NEF-2
-0002
-Soto, M.
-García, L.
-0001</v>
-      </c>
-      <c r="G4" t="str" xml:space="preserve">
-        <v xml:space="preserve">20:00-08:00
-NEF-2
-0001
-García, L.
-Soto, M.
-0002</v>
+        <v>Nacht (vacío en semana 1)</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
       </c>
       <c r="H4" t="str">
         <v/>

</xml_diff>